<commit_message>
Atualização tabela registro + ajuste averbação
</commit_message>
<xml_diff>
--- a/TabelaRegistro.xlsx
+++ b/TabelaRegistro.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Escrituras\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Sistema_Escrituras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE51804-C594-48BD-B2BB-2AAC9870BD6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E06D5F4-5B76-4D6A-9BA2-10BE62349BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>ValorVenal</t>
   </si>
@@ -45,6 +45,12 @@
   </si>
   <si>
     <t>ValorTabela</t>
+  </si>
+  <si>
+    <t>ValorTabelaAv</t>
+  </si>
+  <si>
+    <t>ValorAverbação</t>
   </si>
 </sst>
 </file>
@@ -449,15 +455,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="13.88671875" customWidth="1"/>
     <col min="4" max="4" width="14.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.21875" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -470,8 +478,14 @@
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>2306</v>
       </c>
@@ -482,11 +496,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D2" s="3">
-        <f>SUM(B2:C2)</f>
+        <f t="shared" ref="D2:F23" si="0">SUM(B2:C2)</f>
         <v>343.42</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="3">
+        <v>94.35</v>
+      </c>
+      <c r="F2" s="3">
+        <f>SUM(C2+E2)</f>
+        <v>172.36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>5761</v>
       </c>
@@ -498,11 +519,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D3" s="3">
-        <f>SUM(B3:C3)</f>
+        <f t="shared" si="0"/>
         <v>503.90999999999997</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="3">
+        <v>142.13</v>
+      </c>
+      <c r="F3" s="3">
+        <f>SUM(C3+E3)</f>
+        <v>220.14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>9603</v>
       </c>
@@ -514,11 +542,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D4" s="3">
-        <f>SUM(B4:C4)</f>
+        <f t="shared" si="0"/>
         <v>842.08</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" s="3">
+        <v>242.99</v>
+      </c>
+      <c r="F4" s="3">
+        <f>SUM(C4+E4)</f>
+        <v>321</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>19210</v>
       </c>
@@ -530,11 +565,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D5" s="3">
-        <f>SUM(B5:C5)</f>
+        <f t="shared" si="0"/>
         <v>1211.6600000000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5" s="3">
+        <v>395.7</v>
+      </c>
+      <c r="F5" s="3">
+        <f>SUM(C5+E5)</f>
+        <v>473.71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>38420</v>
       </c>
@@ -546,11 +588,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D6" s="3">
-        <f>SUM(B6:C6)</f>
+        <f t="shared" si="0"/>
         <v>1456.26</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" s="3">
+        <v>504.74</v>
+      </c>
+      <c r="F6" s="3">
+        <f>SUM(C6+E6)</f>
+        <v>582.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>115260</v>
       </c>
@@ -562,11 +611,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D7" s="3">
-        <f>SUM(B7:C7)</f>
+        <f t="shared" si="0"/>
         <v>1615.04</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="3">
+        <v>527.23</v>
+      </c>
+      <c r="F7" s="3">
+        <f>SUM(C7+E7)</f>
+        <v>605.24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>192100</v>
       </c>
@@ -578,11 +634,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D8" s="3">
-        <f>SUM(B8:C8)</f>
+        <f t="shared" si="0"/>
         <v>2039.81</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" s="3">
+        <v>587.23</v>
+      </c>
+      <c r="F8" s="3">
+        <f>SUM(C8+E8)</f>
+        <v>665.24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>230520</v>
       </c>
@@ -594,11 +657,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D9" s="3">
-        <f>SUM(B9:C9)</f>
+        <f t="shared" si="0"/>
         <v>2463.7200000000003</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9" s="3">
+        <v>647.23</v>
+      </c>
+      <c r="F9" s="3">
+        <f>SUM(C9+E9)</f>
+        <v>725.24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>268940</v>
       </c>
@@ -610,11 +680,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D10" s="3">
-        <f>SUM(B10:C10)</f>
+        <f t="shared" si="0"/>
         <v>2675.26</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10" s="3">
+        <v>677.48</v>
+      </c>
+      <c r="F10" s="3">
+        <f>SUM(C10+E10)</f>
+        <v>755.49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>307360</v>
       </c>
@@ -626,11 +703,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D11" s="3">
-        <f>SUM(B11:C11)</f>
+        <f t="shared" si="0"/>
         <v>2887.9900000000002</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" s="3">
+        <v>707.26</v>
+      </c>
+      <c r="F11" s="3">
+        <f>SUM(C11+E11)</f>
+        <v>785.27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>345780</v>
       </c>
@@ -642,11 +726,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D12" s="3">
-        <f>SUM(B12:C12)</f>
+        <f t="shared" si="0"/>
         <v>3040.3</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12" s="3">
+        <v>737.5</v>
+      </c>
+      <c r="F12" s="3">
+        <f>SUM(C12+E12)</f>
+        <v>815.51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>384200</v>
       </c>
@@ -658,11 +749,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D13" s="3">
-        <f>SUM(B13:C13)</f>
+        <f t="shared" si="0"/>
         <v>3117.51</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E13" s="3">
+        <v>767.38</v>
+      </c>
+      <c r="F13" s="3">
+        <f>SUM(C13+E13)</f>
+        <v>845.39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>768400</v>
       </c>
@@ -674,11 +772,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D14" s="3">
-        <f>SUM(B14:C14)</f>
+        <f t="shared" si="0"/>
         <v>3467.0800000000004</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E14" s="3">
+        <v>932.29</v>
+      </c>
+      <c r="F14" s="3">
+        <f>SUM(C14+E14)</f>
+        <v>1010.3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>1152600</v>
       </c>
@@ -690,11 +795,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D15" s="3">
-        <f>SUM(B15:C15)</f>
+        <f t="shared" si="0"/>
         <v>4046.94</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E15" s="3">
+        <v>1232.48</v>
+      </c>
+      <c r="F15" s="3">
+        <f>SUM(C15+E15)</f>
+        <v>1310.49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>1536800</v>
       </c>
@@ -706,11 +818,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D16" s="3">
-        <f>SUM(B16:C16)</f>
+        <f t="shared" si="0"/>
         <v>4647.21</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" s="3">
+        <v>1532.62</v>
+      </c>
+      <c r="F16" s="3">
+        <f>SUM(C16+E16)</f>
+        <v>1610.6299999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>1921000</v>
       </c>
@@ -722,11 +841,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D17" s="3">
-        <f>SUM(B17:C17)</f>
+        <f t="shared" si="0"/>
         <v>5247.5300000000007</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17" s="3">
+        <v>1832.74</v>
+      </c>
+      <c r="F17" s="3">
+        <f>SUM(C17+E17)</f>
+        <v>1910.75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>2305200</v>
       </c>
@@ -738,11 +864,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D18" s="3">
-        <f>SUM(B18:C18)</f>
+        <f t="shared" si="0"/>
         <v>5557.9000000000005</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" s="3">
+        <v>1987.9</v>
+      </c>
+      <c r="F18" s="3">
+        <f>SUM(C18+E18)</f>
+        <v>2065.9100000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>3842000</v>
       </c>
@@ -754,11 +887,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D19" s="3">
-        <f>SUM(B19:C19)</f>
+        <f t="shared" si="0"/>
         <v>7109.6900000000005</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" s="3">
+        <v>2763.8</v>
+      </c>
+      <c r="F19" s="3">
+        <f>SUM(C19+E19)</f>
+        <v>2841.8100000000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>5763000</v>
       </c>
@@ -770,11 +910,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D20" s="3">
-        <f>SUM(B20:C20)</f>
+        <f t="shared" si="0"/>
         <v>9902.89</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E20" s="3">
+        <v>4160.42</v>
+      </c>
+      <c r="F20" s="3">
+        <f>SUM(C20+E20)</f>
+        <v>4238.43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>7684000</v>
       </c>
@@ -786,11 +933,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D21" s="3">
-        <f>SUM(B21:C21)</f>
+        <f t="shared" si="0"/>
         <v>13006.45</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21" s="3">
+        <v>5712.2</v>
+      </c>
+      <c r="F21" s="3">
+        <f>SUM(C21+E21)</f>
+        <v>5790.21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>9605000</v>
       </c>
@@ -802,11 +956,18 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D22" s="3">
-        <f>SUM(B22:C22)</f>
+        <f t="shared" si="0"/>
         <v>16110.02</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22" s="3">
+        <v>7263.98</v>
+      </c>
+      <c r="F22" s="3">
+        <f>SUM(C22+E22)</f>
+        <v>7341.99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>11526000</v>
       </c>
@@ -818,8 +979,15 @@
         <v>78.010000000000005</v>
       </c>
       <c r="D23" s="3">
-        <f>SUM(B23:C23)</f>
+        <f t="shared" si="0"/>
         <v>19213.59</v>
+      </c>
+      <c r="E23" s="3">
+        <v>8815.76</v>
+      </c>
+      <c r="F23" s="3">
+        <f>SUM(C23+E23)</f>
+        <v>8893.77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>